<commit_message>
duy tinh tien loi thang 06 co yen
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="117">
   <si>
     <t>500+1100+2700-105=</t>
   </si>
@@ -372,6 +372,9 @@
   </si>
   <si>
     <t>16/06/2026</t>
+  </si>
+  <si>
+    <t>16/07/2026</t>
   </si>
 </sst>
 </file>
@@ -1449,16 +1452,27 @@
         <v>115</v>
       </c>
     </row>
+    <row r="76" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B76" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C76" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
     <row r="81" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B81" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C81" s="6">
         <f>SUM(C9:C79)</f>
-        <v>89805</v>
+        <v>92805</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="85" spans="2:4" ht="21" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
duy tinh tien loi thang 07 co yen
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="118">
   <si>
     <t>500+1100+2700-105=</t>
   </si>
@@ -375,6 +375,9 @@
   </si>
   <si>
     <t>16/07/2026</t>
+  </si>
+  <si>
+    <t>16/08/2026</t>
   </si>
 </sst>
 </file>
@@ -1463,16 +1466,27 @@
         <v>116</v>
       </c>
     </row>
+    <row r="77" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B77" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C77" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
     <row r="81" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B81" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C81" s="6">
         <f>SUM(C9:C79)</f>
-        <v>92805</v>
+        <v>95805</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="85" spans="2:4" ht="21" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
tinh tien loi co yen thang 08
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="119">
   <si>
     <t>500+1100+2700-105=</t>
   </si>
@@ -378,6 +378,9 @@
   </si>
   <si>
     <t>16/08/2026</t>
+  </si>
+  <si>
+    <t>16/09/2026</t>
   </si>
 </sst>
 </file>
@@ -712,7 +715,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:D156"/>
+  <dimension ref="A2:D157"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" style="1" customWidth="1"/>
@@ -1477,24 +1480,35 @@
         <v>117</v>
       </c>
     </row>
-    <row r="81" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B81" s="5" t="s">
+    <row r="78" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B78" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C78" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="82" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B82" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C81" s="6">
-        <f>SUM(C9:C79)</f>
-        <v>95805</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="85" spans="2:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="B85" s="5"/>
-      <c r="C85" s="7"/>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A156" s="2"/>
+      <c r="C82" s="6">
+        <f>SUM(C9:C80)</f>
+        <v>98805</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="86" spans="2:4" ht="21" x14ac:dyDescent="0.35">
+      <c r="B86" s="5"/>
+      <c r="C86" s="7"/>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
duy tinh tien loi thang 09 co yen
</commit_message>
<xml_diff>
--- a/ThuChiCoYenLinhTrung.xlsx
+++ b/ThuChiCoYenLinhTrung.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="120">
   <si>
     <t>500+1100+2700-105=</t>
   </si>
@@ -381,6 +381,9 @@
   </si>
   <si>
     <t>16/09/2026</t>
+  </si>
+  <si>
+    <t>16/10/2026</t>
   </si>
 </sst>
 </file>
@@ -715,7 +718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:D157"/>
+  <dimension ref="A2:D159"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" style="1" customWidth="1"/>
@@ -1491,24 +1494,35 @@
         <v>118</v>
       </c>
     </row>
-    <row r="82" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B82" s="5" t="s">
+    <row r="79" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B79" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C79" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="84" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B84" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C82" s="6">
-        <f>SUM(C9:C80)</f>
-        <v>98805</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="86" spans="2:4" ht="21" x14ac:dyDescent="0.35">
-      <c r="B86" s="5"/>
-      <c r="C86" s="7"/>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A157" s="2"/>
+      <c r="C84" s="6">
+        <f>SUM(C9:C82)</f>
+        <v>101805</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="88" spans="2:4" ht="21" x14ac:dyDescent="0.35">
+      <c r="B88" s="5"/>
+      <c r="C88" s="7"/>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>